<commit_message>
Minimal updates to BOM
</commit_message>
<xml_diff>
--- a/Walking-Setup/G6-Integration-Bill-of-Materials.xlsx
+++ b/Walking-Setup/G6-Integration-Bill-of-Materials.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10703"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lehenbaueri/Documents/GitHub/Fly-Lab-Gear/Walking-Setup/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50363D00-03FF-BB4E-9D05-0301A7584635}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A04A191-27BF-7F49-95A7-8C52F28F758E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6460" yWindow="1600" windowWidth="27460" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1640" yWindow="660" windowWidth="27460" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,15 +33,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="152">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="306" uniqueCount="151">
   <si>
     <t>Name</t>
   </si>
   <si>
     <t>G6 Fly on Ball Walking Setup</t>
-  </si>
-  <si>
-    <t>Number</t>
   </si>
   <si>
     <t>Revision</t>
@@ -551,7 +548,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -563,7 +560,6 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
@@ -621,8 +617,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A10:K63" totalsRowShown="0">
-  <autoFilter ref="A10:K63" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A9:K62" totalsRowShown="0">
+  <autoFilter ref="A9:K62" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="11">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Category"/>
     <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Subassembly"/>
@@ -959,7 +955,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K63"/>
+  <dimension ref="A1:K62"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -985,20 +981,20 @@
       <c r="A2" s="2" t="s">
         <v>2</v>
       </c>
+      <c r="B2">
+        <v>2</v>
+      </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B3">
-        <v>2</v>
+      <c r="B3" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4" t="s">
         <v>5</v>
       </c>
     </row>
@@ -1006,239 +1002,256 @@
       <c r="A5" s="2" t="s">
         <v>6</v>
       </c>
+      <c r="B5">
+        <f>SUM(Table1[Qty])</f>
+        <v>104.5</v>
+      </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B6">
-        <f>SUM(Table1[Qty])</f>
-        <v>104.5</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A7" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B7" s="3">
+      <c r="B6" s="3">
         <f>SUM(Table1[Cost])</f>
         <v>588.54019999999991</v>
       </c>
     </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>9</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="D9" t="s">
+        <v>11</v>
+      </c>
+      <c r="E9" t="s">
+        <v>12</v>
+      </c>
+      <c r="F9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G9" t="s">
+        <v>14</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="I9" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="J9" t="s">
+        <v>17</v>
+      </c>
+      <c r="K9" t="s">
+        <v>18</v>
+      </c>
+    </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
-        <v>9</v>
-      </c>
-      <c r="B10" t="s">
-        <v>10</v>
-      </c>
       <c r="C10" s="5" t="s">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="D10" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="E10" t="s">
-        <v>13</v>
-      </c>
-      <c r="F10" t="s">
-        <v>14</v>
-      </c>
-      <c r="G10" t="s">
-        <v>15</v>
-      </c>
-      <c r="H10" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="I10" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="J10" t="s">
-        <v>18</v>
-      </c>
-      <c r="K10" t="s">
-        <v>19</v>
+        <v>21</v>
+      </c>
+      <c r="F10">
+        <v>1</v>
+      </c>
+      <c r="G10" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="H10" s="1">
+        <v>184.47</v>
+      </c>
+      <c r="I10" s="1">
+        <f>Table1[[#This Row],[Qty]]*Table1[[#This Row],[Unit Cost]]</f>
+        <v>184.47</v>
+      </c>
+      <c r="J10" s="4" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="C11" s="5" t="s">
-        <v>20</v>
+      <c r="B11" t="s">
+        <v>24</v>
       </c>
       <c r="D11" t="s">
-        <v>21</v>
-      </c>
-      <c r="E11" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="F11">
         <v>1</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="H11" s="1">
-        <v>184.47</v>
+        <v>22</v>
       </c>
       <c r="I11" s="1">
         <f>Table1[[#This Row],[Qty]]*Table1[[#This Row],[Unit Cost]]</f>
-        <v>184.47</v>
+        <v>0</v>
       </c>
       <c r="J11" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B12" t="s">
-        <v>25</v>
+        <v>24</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>26</v>
       </c>
       <c r="D12" t="s">
-        <v>25</v>
+        <v>27</v>
+      </c>
+      <c r="E12" t="s">
+        <v>21</v>
       </c>
       <c r="F12">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
+      </c>
+      <c r="H12" s="1">
+        <v>5.76</v>
       </c>
       <c r="I12" s="1">
         <f>Table1[[#This Row],[Qty]]*Table1[[#This Row],[Unit Cost]]</f>
-        <v>0</v>
+        <v>23.04</v>
       </c>
       <c r="J12" s="4" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>29</v>
+      </c>
       <c r="B13" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="D13" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="E13" t="s">
-        <v>22</v>
+        <v>32</v>
       </c>
       <c r="F13">
         <v>4</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="H13" s="1">
-        <v>5.76</v>
+        <f>14.44/100</f>
+        <v>0.1444</v>
       </c>
       <c r="I13" s="1">
         <f>Table1[[#This Row],[Qty]]*Table1[[#This Row],[Unit Cost]]</f>
-        <v>23.04</v>
+        <v>0.5776</v>
       </c>
       <c r="J13" s="4" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B14" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="D14" t="s">
+        <v>35</v>
+      </c>
+      <c r="E14" t="s">
         <v>32</v>
       </c>
-      <c r="E14" t="s">
-        <v>33</v>
-      </c>
       <c r="F14">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="H14" s="1">
-        <f>14.44/100</f>
-        <v>0.1444</v>
-      </c>
-      <c r="I14" s="1">
-        <f>Table1[[#This Row],[Qty]]*Table1[[#This Row],[Unit Cost]]</f>
-        <v>0.5776</v>
-      </c>
-      <c r="J14" s="4" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A15" t="s">
-        <v>30</v>
-      </c>
-      <c r="B15" t="s">
-        <v>25</v>
-      </c>
-      <c r="C15" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="D15" t="s">
-        <v>36</v>
-      </c>
-      <c r="E15" t="s">
-        <v>33</v>
-      </c>
-      <c r="F15">
-        <v>8</v>
-      </c>
-      <c r="G15" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="H15" s="1">
         <f>2.02/100</f>
         <v>2.0199999999999999E-2</v>
       </c>
+      <c r="I14" s="1">
+        <f>Table1[[#This Row],[Qty]]*Table1[[#This Row],[Unit Cost]]</f>
+        <v>0.16159999999999999</v>
+      </c>
+      <c r="J14" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="B15" t="s">
+        <v>24</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="D15" t="s">
+        <v>38</v>
+      </c>
+      <c r="E15" t="s">
+        <v>39</v>
+      </c>
+      <c r="F15">
+        <v>4</v>
+      </c>
+      <c r="G15" s="5" t="s">
+        <v>40</v>
+      </c>
       <c r="I15" s="1">
         <f>Table1[[#This Row],[Qty]]*Table1[[#This Row],[Unit Cost]]</f>
-        <v>0.16159999999999999</v>
+        <v>0</v>
       </c>
       <c r="J15" s="4" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>42</v>
+      </c>
       <c r="B16" t="s">
-        <v>25</v>
-      </c>
-      <c r="C16" s="5" t="s">
-        <v>38</v>
+        <v>24</v>
       </c>
       <c r="D16" t="s">
-        <v>39</v>
-      </c>
-      <c r="E16" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="F16">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>41</v>
+        <v>22</v>
       </c>
       <c r="I16" s="1">
         <f>Table1[[#This Row],[Qty]]*Table1[[#This Row],[Unit Cost]]</f>
         <v>0</v>
       </c>
-      <c r="J16" s="4" t="s">
-        <v>42</v>
-      </c>
+      <c r="J16" s="4"/>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B17" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D17" t="s">
         <v>44</v>
@@ -1247,250 +1260,247 @@
         <v>1</v>
       </c>
       <c r="G17" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
+      </c>
+      <c r="H17" s="1">
+        <v>4.5</v>
       </c>
       <c r="I17" s="1">
         <f>Table1[[#This Row],[Qty]]*Table1[[#This Row],[Unit Cost]]</f>
-        <v>0</v>
-      </c>
-      <c r="J17" s="4"/>
+        <v>4.5</v>
+      </c>
+      <c r="J17" s="4" t="s">
+        <v>45</v>
+      </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>43</v>
+        <v>29</v>
       </c>
       <c r="B18" t="s">
-        <v>25</v>
+        <v>46</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>47</v>
       </c>
       <c r="D18" t="s">
-        <v>45</v>
+        <v>48</v>
+      </c>
+      <c r="E18" t="s">
+        <v>32</v>
       </c>
       <c r="F18">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G18" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="H18" s="1">
-        <v>4.5</v>
+        <f>13.88/25</f>
+        <v>0.55520000000000003</v>
       </c>
       <c r="I18" s="1">
         <f>Table1[[#This Row],[Qty]]*Table1[[#This Row],[Unit Cost]]</f>
-        <v>4.5</v>
+        <v>2.2208000000000001</v>
       </c>
       <c r="J18" s="4" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B19" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>48</v>
+        <v>34</v>
       </c>
       <c r="D19" t="s">
-        <v>49</v>
+        <v>35</v>
       </c>
       <c r="E19" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F19">
         <v>4</v>
       </c>
       <c r="G19" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="H19" s="1">
-        <f>13.88/25</f>
-        <v>0.55520000000000003</v>
+        <v>0.02</v>
       </c>
       <c r="I19" s="1">
         <f>Table1[[#This Row],[Qty]]*Table1[[#This Row],[Unit Cost]]</f>
-        <v>2.2208000000000001</v>
+        <v>0.08</v>
       </c>
       <c r="J19" s="4" t="s">
-        <v>50</v>
+        <v>36</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B20" t="s">
-        <v>47</v>
+        <v>24</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>35</v>
+        <v>50</v>
       </c>
       <c r="D20" t="s">
-        <v>36</v>
+        <v>51</v>
       </c>
       <c r="E20" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F20">
         <v>4</v>
       </c>
       <c r="G20" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="H20" s="1">
-        <v>0.02</v>
-      </c>
-      <c r="I20" s="1">
-        <f>Table1[[#This Row],[Qty]]*Table1[[#This Row],[Unit Cost]]</f>
-        <v>0.08</v>
-      </c>
-      <c r="J20" s="4" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A21" t="s">
-        <v>30</v>
-      </c>
-      <c r="B21" t="s">
-        <v>25</v>
-      </c>
-      <c r="C21" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="D21" t="s">
-        <v>52</v>
-      </c>
-      <c r="E21" t="s">
-        <v>33</v>
-      </c>
-      <c r="F21">
-        <v>4</v>
-      </c>
-      <c r="G21" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="H21" s="1">
         <f>14.83/100</f>
         <v>0.14829999999999999</v>
       </c>
+      <c r="I20" s="1">
+        <f>Table1[[#This Row],[Qty]]*Table1[[#This Row],[Unit Cost]]</f>
+        <v>0.59319999999999995</v>
+      </c>
+      <c r="J20" s="4" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="B21" t="s">
+        <v>46</v>
+      </c>
+      <c r="C21" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="D21" t="s">
+        <v>54</v>
+      </c>
+      <c r="E21" t="s">
+        <v>32</v>
+      </c>
+      <c r="F21">
+        <v>1</v>
+      </c>
+      <c r="G21" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="H21" s="1">
+        <v>2.89</v>
+      </c>
       <c r="I21" s="1">
         <f>Table1[[#This Row],[Qty]]*Table1[[#This Row],[Unit Cost]]</f>
-        <v>0.59319999999999995</v>
+        <v>2.89</v>
       </c>
       <c r="J21" s="4" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B22" t="s">
-        <v>47</v>
-      </c>
-      <c r="C22" s="5" t="s">
-        <v>54</v>
+        <v>46</v>
       </c>
       <c r="D22" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E22" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="F22">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G22" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="H22" s="1">
-        <v>2.89</v>
+        <v>22</v>
       </c>
       <c r="I22" s="1">
         <f>Table1[[#This Row],[Qty]]*Table1[[#This Row],[Unit Cost]]</f>
-        <v>2.89</v>
+        <v>0</v>
       </c>
       <c r="J22" s="4" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B23" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D23" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E23" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F23">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G23" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="I23" s="1">
         <f>Table1[[#This Row],[Qty]]*Table1[[#This Row],[Unit Cost]]</f>
         <v>0</v>
       </c>
       <c r="J23" s="4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B24" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D24" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E24" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F24">
         <v>1</v>
       </c>
       <c r="G24" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="I24" s="1">
         <f>Table1[[#This Row],[Qty]]*Table1[[#This Row],[Unit Cost]]</f>
         <v>0</v>
       </c>
       <c r="J24" s="4" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>42</v>
+      </c>
       <c r="B25" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D25" t="s">
-        <v>61</v>
-      </c>
-      <c r="E25" t="s">
-        <v>40</v>
+        <v>62</v>
       </c>
       <c r="F25">
         <v>1</v>
       </c>
       <c r="G25" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="I25" s="1">
-        <f>Table1[[#This Row],[Qty]]*Table1[[#This Row],[Unit Cost]]</f>
-        <v>0</v>
-      </c>
-      <c r="J25" s="4" t="s">
-        <v>62</v>
-      </c>
+        <v>22</v>
+      </c>
+      <c r="I25" s="1"/>
+      <c r="J25" s="4"/>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B26" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D26" t="s">
         <v>63</v>
@@ -1498,16 +1508,18 @@
       <c r="F26">
         <v>1</v>
       </c>
-      <c r="G26" s="5"/>
+      <c r="G26" s="5" t="s">
+        <v>22</v>
+      </c>
       <c r="I26" s="1"/>
       <c r="J26" s="4"/>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B27" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D27" t="s">
         <v>64</v>
@@ -1515,1015 +1527,998 @@
       <c r="F27">
         <v>1</v>
       </c>
-      <c r="G27" s="5"/>
+      <c r="G27" s="5" t="s">
+        <v>22</v>
+      </c>
       <c r="I27" s="1"/>
       <c r="J27" s="4"/>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A28" t="s">
-        <v>43</v>
-      </c>
       <c r="B28" t="s">
-        <v>47</v>
+        <v>46</v>
+      </c>
+      <c r="C28" s="5" t="s">
+        <v>65</v>
       </c>
       <c r="D28" t="s">
-        <v>65</v>
+        <v>66</v>
+      </c>
+      <c r="E28" t="s">
+        <v>67</v>
       </c>
       <c r="F28">
         <v>1</v>
       </c>
       <c r="G28" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="I28" s="1"/>
-      <c r="J28" s="4"/>
+        <v>22</v>
+      </c>
+      <c r="H28" s="1">
+        <v>11.34</v>
+      </c>
+      <c r="I28" s="1">
+        <f>Table1[[#This Row],[Qty]]*Table1[[#This Row],[Unit Cost]]</f>
+        <v>11.34</v>
+      </c>
+      <c r="J28" s="4" t="s">
+        <v>68</v>
+      </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B29" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="D29" t="s">
+        <v>70</v>
+      </c>
+      <c r="E29" t="s">
         <v>67</v>
       </c>
-      <c r="E29" t="s">
-        <v>68</v>
-      </c>
       <c r="F29">
         <v>1</v>
       </c>
       <c r="G29" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="H29" s="1">
-        <v>11.34</v>
+        <v>5.14</v>
       </c>
       <c r="I29" s="1">
         <f>Table1[[#This Row],[Qty]]*Table1[[#This Row],[Unit Cost]]</f>
-        <v>11.34</v>
-      </c>
-      <c r="J29" s="4" t="s">
-        <v>69</v>
+        <v>5.14</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B30" t="s">
-        <v>47</v>
-      </c>
-      <c r="C30" s="5" t="s">
-        <v>70</v>
+        <v>46</v>
+      </c>
+      <c r="C30" s="5">
+        <v>10193</v>
       </c>
       <c r="D30" t="s">
         <v>71</v>
       </c>
       <c r="E30" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="F30">
         <v>1</v>
       </c>
       <c r="G30" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="H30" s="1">
-        <v>5.14</v>
+        <v>1.71</v>
       </c>
       <c r="I30" s="1">
         <f>Table1[[#This Row],[Qty]]*Table1[[#This Row],[Unit Cost]]</f>
-        <v>5.14</v>
+        <v>1.71</v>
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A31" t="s">
+        <v>29</v>
+      </c>
       <c r="B31" t="s">
-        <v>47</v>
-      </c>
-      <c r="C31" s="5">
-        <v>10193</v>
+        <v>46</v>
+      </c>
+      <c r="C31" s="5" t="s">
+        <v>72</v>
       </c>
       <c r="D31" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="E31" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="F31">
         <v>1</v>
       </c>
       <c r="G31" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="H31" s="1">
-        <v>1.71</v>
+        <v>1.92</v>
       </c>
       <c r="I31" s="1">
         <f>Table1[[#This Row],[Qty]]*Table1[[#This Row],[Unit Cost]]</f>
-        <v>1.71</v>
+        <v>1.92</v>
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="B32" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D32" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E32" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="F32">
         <v>1</v>
       </c>
       <c r="G32" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="H32" s="1">
-        <v>1.92</v>
+        <v>17.239999999999998</v>
       </c>
       <c r="I32" s="1">
         <f>Table1[[#This Row],[Qty]]*Table1[[#This Row],[Unit Cost]]</f>
-        <v>1.92</v>
+        <v>17.239999999999998</v>
       </c>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B33" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D33" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E33" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="F33">
         <v>1</v>
       </c>
       <c r="G33" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="H33" s="1">
-        <v>17.239999999999998</v>
+        <v>2.56</v>
       </c>
       <c r="I33" s="1">
         <f>Table1[[#This Row],[Qty]]*Table1[[#This Row],[Unit Cost]]</f>
-        <v>17.239999999999998</v>
+        <v>2.56</v>
       </c>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B34" t="s">
-        <v>47</v>
-      </c>
-      <c r="C34" s="5" t="s">
-        <v>77</v>
+        <v>46</v>
       </c>
       <c r="D34" t="s">
         <v>78</v>
       </c>
-      <c r="E34" t="s">
-        <v>68</v>
-      </c>
       <c r="F34">
         <v>1</v>
       </c>
       <c r="G34" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="H34" s="1">
-        <v>2.56</v>
+        <v>22</v>
       </c>
       <c r="I34" s="1">
         <f>Table1[[#This Row],[Qty]]*Table1[[#This Row],[Unit Cost]]</f>
-        <v>2.56</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A35" t="s">
-        <v>43</v>
-      </c>
       <c r="B35" t="s">
-        <v>47</v>
+        <v>79</v>
       </c>
       <c r="D35" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F35">
         <v>1</v>
       </c>
       <c r="G35" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
+      </c>
+      <c r="H35" s="1">
+        <v>80</v>
       </c>
       <c r="I35" s="1">
         <f>Table1[[#This Row],[Qty]]*Table1[[#This Row],[Unit Cost]]</f>
-        <v>0</v>
+        <v>80</v>
       </c>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B36" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D36" t="s">
         <v>81</v>
       </c>
+      <c r="E36" t="s">
+        <v>39</v>
+      </c>
       <c r="F36">
         <v>1</v>
       </c>
       <c r="G36" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="H36" s="1">
-        <v>80</v>
+        <v>22</v>
       </c>
       <c r="I36" s="1">
         <f>Table1[[#This Row],[Qty]]*Table1[[#This Row],[Unit Cost]]</f>
-        <v>80</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B37" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D37" t="s">
         <v>82</v>
       </c>
       <c r="E37" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F37">
         <v>1</v>
       </c>
       <c r="G37" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="I37" s="1">
         <f>Table1[[#This Row],[Qty]]*Table1[[#This Row],[Unit Cost]]</f>
         <v>0</v>
+      </c>
+      <c r="J37" s="6" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B38" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D38" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="E38" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F38">
         <v>1</v>
       </c>
       <c r="G38" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="I38" s="1">
         <f>Table1[[#This Row],[Qty]]*Table1[[#This Row],[Unit Cost]]</f>
         <v>0</v>
       </c>
       <c r="J38" s="6" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B39" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D39" t="s">
-        <v>85</v>
-      </c>
-      <c r="E39" t="s">
-        <v>40</v>
+        <v>86</v>
       </c>
       <c r="F39">
         <v>1</v>
       </c>
       <c r="G39" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="I39" s="1">
         <f>Table1[[#This Row],[Qty]]*Table1[[#This Row],[Unit Cost]]</f>
         <v>0</v>
       </c>
-      <c r="J39" s="6" t="s">
-        <v>86</v>
-      </c>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A40" t="s">
+        <v>29</v>
+      </c>
       <c r="B40" t="s">
-        <v>80</v>
+        <v>79</v>
+      </c>
+      <c r="C40" s="5" t="s">
+        <v>87</v>
       </c>
       <c r="D40" t="s">
-        <v>87</v>
+        <v>88</v>
+      </c>
+      <c r="E40" t="s">
+        <v>32</v>
       </c>
       <c r="F40">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G40" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
+      </c>
+      <c r="H40" s="1">
+        <f>17.78/100</f>
+        <v>0.17780000000000001</v>
       </c>
       <c r="I40" s="1">
         <f>Table1[[#This Row],[Qty]]*Table1[[#This Row],[Unit Cost]]</f>
-        <v>0</v>
+        <v>0.88900000000000001</v>
+      </c>
+      <c r="J40" s="4" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B41" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C41" s="5" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="D41" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="E41" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F41">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G41" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="H41" s="1">
-        <f>17.78/100</f>
-        <v>0.17780000000000001</v>
+        <f>3.06/100</f>
+        <v>3.0600000000000002E-2</v>
       </c>
       <c r="I41" s="1">
         <f>Table1[[#This Row],[Qty]]*Table1[[#This Row],[Unit Cost]]</f>
-        <v>0.88900000000000001</v>
+        <v>3.0600000000000002E-2</v>
       </c>
       <c r="J41" s="4" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>30</v>
+        <v>93</v>
       </c>
       <c r="B42" t="s">
-        <v>80</v>
+        <v>93</v>
       </c>
       <c r="C42" s="5" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="D42" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="E42" t="s">
-        <v>33</v>
+        <v>96</v>
       </c>
       <c r="F42">
         <v>1</v>
       </c>
       <c r="G42" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="H42" s="1">
+        <v>229</v>
+      </c>
+      <c r="I42" s="1">
+        <f>Table1[[#This Row],[Qty]]*Table1[[#This Row],[Unit Cost]]</f>
+        <v>229</v>
+      </c>
+      <c r="J42" s="4" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="43" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="B43" t="s">
+        <v>93</v>
+      </c>
+      <c r="D43" t="s">
+        <v>98</v>
+      </c>
+      <c r="F43">
+        <v>1</v>
+      </c>
+      <c r="G43" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="I43" s="1">
+        <f>Table1[[#This Row],[Qty]]*Table1[[#This Row],[Unit Cost]]</f>
+        <v>0</v>
+      </c>
+      <c r="J43" s="4"/>
+    </row>
+    <row r="44" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A44" t="s">
+        <v>29</v>
+      </c>
+      <c r="B44" t="s">
+        <v>93</v>
+      </c>
+      <c r="C44" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="D44" t="s">
+        <v>100</v>
+      </c>
+      <c r="E44" t="s">
+        <v>32</v>
+      </c>
+      <c r="F44">
+        <v>6</v>
+      </c>
+      <c r="G44" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="H44" s="1">
+        <f>17.63/100</f>
+        <v>0.17629999999999998</v>
+      </c>
+      <c r="I44" s="1">
+        <f>Table1[[#This Row],[Qty]]*Table1[[#This Row],[Unit Cost]]</f>
+        <v>1.0577999999999999</v>
+      </c>
+      <c r="J44" s="4" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="45" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A45" t="s">
+        <v>29</v>
+      </c>
+      <c r="B45" t="s">
+        <v>93</v>
+      </c>
+      <c r="C45" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="D45" t="s">
+        <v>103</v>
+      </c>
+      <c r="E45" t="s">
+        <v>32</v>
+      </c>
+      <c r="F45">
+        <v>6</v>
+      </c>
+      <c r="G45" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="H45" s="1">
+        <f>3/100</f>
+        <v>0.03</v>
+      </c>
+      <c r="I45" s="1">
+        <f>Table1[[#This Row],[Qty]]*Table1[[#This Row],[Unit Cost]]</f>
+        <v>0.18</v>
+      </c>
+      <c r="J45" s="4" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="46" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="B46" t="s">
+        <v>93</v>
+      </c>
+      <c r="D46" t="s">
+        <v>105</v>
+      </c>
+      <c r="F46">
+        <v>1</v>
+      </c>
+      <c r="G46" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="H46" s="1">
+        <v>5</v>
+      </c>
+      <c r="I46" s="1">
+        <f>Table1[[#This Row],[Qty]]*Table1[[#This Row],[Unit Cost]]</f>
+        <v>5</v>
+      </c>
+      <c r="J46" s="4" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="47" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A47" t="s">
+        <v>42</v>
+      </c>
+      <c r="B47" t="s">
+        <v>107</v>
+      </c>
+      <c r="D47" t="s">
+        <v>108</v>
+      </c>
+      <c r="E47" t="s">
+        <v>109</v>
+      </c>
+      <c r="F47">
+        <v>1</v>
+      </c>
+      <c r="G47" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="H47" s="1">
+        <v>0</v>
+      </c>
+      <c r="I47" s="1">
+        <f>Table1[[#This Row],[Qty]]*Table1[[#This Row],[Unit Cost]]</f>
+        <v>0</v>
+      </c>
+      <c r="J47" s="6" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="48" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A48" t="s">
+        <v>29</v>
+      </c>
+      <c r="B48" t="s">
+        <v>107</v>
+      </c>
+      <c r="D48" t="s">
+        <v>111</v>
+      </c>
+      <c r="E48" t="s">
+        <v>32</v>
+      </c>
+      <c r="F48">
+        <v>2</v>
+      </c>
+      <c r="G48" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="H48" s="1">
+        <f>11.38/50</f>
+        <v>0.22760000000000002</v>
+      </c>
+      <c r="I48" s="1">
+        <f>Table1[[#This Row],[Qty]]*Table1[[#This Row],[Unit Cost]]</f>
+        <v>0.45520000000000005</v>
+      </c>
+      <c r="J48" s="4" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="49" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="B49" t="s">
+        <v>107</v>
+      </c>
+      <c r="D49" t="s">
+        <v>113</v>
+      </c>
+      <c r="E49" t="s">
+        <v>114</v>
+      </c>
+      <c r="F49">
+        <v>1</v>
+      </c>
+      <c r="G49" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="I49" s="1">
+        <f>Table1[[#This Row],[Qty]]*Table1[[#This Row],[Unit Cost]]</f>
+        <v>0</v>
+      </c>
+      <c r="J49" s="4" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="50" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="B50" t="s">
+        <v>107</v>
+      </c>
+      <c r="D50" t="s">
+        <v>116</v>
+      </c>
+      <c r="F50">
+        <v>1</v>
+      </c>
+      <c r="G50" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="I50" s="1">
+        <f>Table1[[#This Row],[Qty]]*Table1[[#This Row],[Unit Cost]]</f>
+        <v>0</v>
+      </c>
+      <c r="J50" s="6" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A51" t="s">
+        <v>29</v>
+      </c>
+      <c r="B51" t="s">
+        <v>107</v>
+      </c>
+      <c r="C51" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="D51" t="s">
+        <v>119</v>
+      </c>
+      <c r="E51" t="s">
+        <v>32</v>
+      </c>
+      <c r="F51">
+        <v>3</v>
+      </c>
+      <c r="G51" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="H51" s="1">
+        <f>7.57/100</f>
+        <v>7.5700000000000003E-2</v>
+      </c>
+      <c r="I51" s="1">
+        <f>Table1[[#This Row],[Qty]]*Table1[[#This Row],[Unit Cost]]</f>
+        <v>0.22710000000000002</v>
+      </c>
+      <c r="J51" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="52" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A52" t="s">
+        <v>29</v>
+      </c>
+      <c r="B52" t="s">
+        <v>107</v>
+      </c>
+      <c r="C52" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="D52" t="s">
+        <v>122</v>
+      </c>
+      <c r="E52" t="s">
+        <v>32</v>
+      </c>
+      <c r="F52">
+        <v>3</v>
+      </c>
+      <c r="G52" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="H52" s="1">
+        <f>7.41/100</f>
+        <v>7.4099999999999999E-2</v>
+      </c>
+      <c r="I52" s="1">
+        <f>Table1[[#This Row],[Qty]]*Table1[[#This Row],[Unit Cost]]</f>
+        <v>0.2223</v>
+      </c>
+      <c r="J52" s="4" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="53" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="B53" t="s">
+        <v>107</v>
+      </c>
+      <c r="C53" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="D53" t="s">
+        <v>149</v>
+      </c>
+      <c r="E53" t="s">
+        <v>32</v>
+      </c>
+      <c r="F53">
+        <v>1</v>
+      </c>
+      <c r="G53" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="H53" s="1">
+        <v>4.95</v>
+      </c>
+      <c r="I53" s="1">
+        <f>Table1[[#This Row],[Qty]]*Table1[[#This Row],[Unit Cost]]</f>
+        <v>4.95</v>
+      </c>
+      <c r="J53" s="4" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="54" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="B54" t="s">
+        <v>124</v>
+      </c>
+      <c r="D54" t="s">
+        <v>125</v>
+      </c>
+      <c r="G54" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="I54" s="1">
+        <f>Table1[[#This Row],[Qty]]*Table1[[#This Row],[Unit Cost]]</f>
+        <v>0</v>
+      </c>
+      <c r="J54" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="55" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="B55" t="s">
+        <v>124</v>
+      </c>
+      <c r="D55" t="s">
+        <v>127</v>
+      </c>
+      <c r="F55">
+        <v>1</v>
+      </c>
+      <c r="G55" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="I55" s="1">
+        <f>Table1[[#This Row],[Qty]]*Table1[[#This Row],[Unit Cost]]</f>
+        <v>0</v>
+      </c>
+      <c r="J55" s="6" t="s">
+        <v>128</v>
+      </c>
+      <c r="K55" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="56" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="B56" t="s">
+        <v>124</v>
+      </c>
+      <c r="C56" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="D56" t="s">
+        <v>131</v>
+      </c>
+      <c r="E56" t="s">
+        <v>132</v>
+      </c>
+      <c r="F56">
+        <v>1</v>
+      </c>
+      <c r="G56" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="H56" s="1">
+        <v>1.08</v>
+      </c>
+      <c r="I56" s="1">
+        <f>Table1[[#This Row],[Qty]]*Table1[[#This Row],[Unit Cost]]</f>
+        <v>1.08</v>
+      </c>
+      <c r="J56" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="57" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="B57" t="s">
+        <v>124</v>
+      </c>
+      <c r="D57" t="s">
+        <v>134</v>
+      </c>
+      <c r="G57" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="I57" s="1">
+        <f>Table1[[#This Row],[Qty]]*Table1[[#This Row],[Unit Cost]]</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A58" t="s">
+        <v>42</v>
+      </c>
+      <c r="B58" t="s">
+        <v>135</v>
+      </c>
+      <c r="C58" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="D58" t="s">
+        <v>137</v>
+      </c>
+      <c r="E58" t="s">
+        <v>67</v>
+      </c>
+      <c r="F58">
+        <v>1</v>
+      </c>
+      <c r="G58" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="H58" s="1">
+        <v>1.49</v>
+      </c>
+      <c r="I58" s="1">
+        <f>Table1[[#This Row],[Qty]]*Table1[[#This Row],[Unit Cost]]</f>
+        <v>1.49</v>
+      </c>
+      <c r="J58" s="4" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="59" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A59" t="s">
+        <v>29</v>
+      </c>
+      <c r="B59" t="s">
+        <v>135</v>
+      </c>
+      <c r="C59" s="5" t="s">
+        <v>139</v>
+      </c>
+      <c r="D59" t="s">
+        <v>140</v>
+      </c>
+      <c r="E59" t="s">
+        <v>32</v>
+      </c>
+      <c r="F59">
+        <v>6</v>
+      </c>
+      <c r="G59" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="H59" s="1">
+        <f>8.44/100</f>
+        <v>8.4399999999999989E-2</v>
+      </c>
+      <c r="I59" s="1">
+        <f>Table1[[#This Row],[Qty]]*Table1[[#This Row],[Unit Cost]]</f>
+        <v>0.50639999999999996</v>
+      </c>
+      <c r="J59" s="4" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="60" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A60" t="s">
+        <v>29</v>
+      </c>
+      <c r="B60" t="s">
+        <v>135</v>
+      </c>
+      <c r="C60" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="D60" t="s">
+        <v>142</v>
+      </c>
+      <c r="E60" t="s">
+        <v>32</v>
+      </c>
+      <c r="F60">
+        <v>6</v>
+      </c>
+      <c r="G60" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="H60" s="1">
         <f>3.06/100</f>
         <v>3.0600000000000002E-2</v>
       </c>
-      <c r="I42" s="1">
-        <f>Table1[[#This Row],[Qty]]*Table1[[#This Row],[Unit Cost]]</f>
-        <v>3.0600000000000002E-2</v>
-      </c>
-      <c r="J42" s="4" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A43" t="s">
-        <v>94</v>
-      </c>
-      <c r="B43" t="s">
-        <v>94</v>
-      </c>
-      <c r="C43" s="5" t="s">
-        <v>95</v>
-      </c>
-      <c r="D43" t="s">
-        <v>96</v>
-      </c>
-      <c r="E43" t="s">
-        <v>97</v>
-      </c>
-      <c r="F43">
-        <v>1</v>
-      </c>
-      <c r="G43" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="H43" s="1">
-        <v>229</v>
-      </c>
-      <c r="I43" s="1">
-        <f>Table1[[#This Row],[Qty]]*Table1[[#This Row],[Unit Cost]]</f>
-        <v>229</v>
-      </c>
-      <c r="J43" s="4" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="B44" t="s">
-        <v>94</v>
-      </c>
-      <c r="D44" t="s">
-        <v>99</v>
-      </c>
-      <c r="F44">
-        <v>1</v>
-      </c>
-      <c r="G44" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="I44" s="1">
-        <f>Table1[[#This Row],[Qty]]*Table1[[#This Row],[Unit Cost]]</f>
-        <v>0</v>
-      </c>
-      <c r="J44" s="4"/>
-    </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A45" t="s">
-        <v>30</v>
-      </c>
-      <c r="B45" t="s">
-        <v>94</v>
-      </c>
-      <c r="C45" s="5" t="s">
-        <v>100</v>
-      </c>
-      <c r="D45" t="s">
-        <v>101</v>
-      </c>
-      <c r="E45" t="s">
-        <v>33</v>
-      </c>
-      <c r="F45">
-        <v>6</v>
-      </c>
-      <c r="G45" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="H45" s="1">
-        <f>17.63/100</f>
-        <v>0.17629999999999998</v>
-      </c>
-      <c r="I45" s="1">
-        <f>Table1[[#This Row],[Qty]]*Table1[[#This Row],[Unit Cost]]</f>
-        <v>1.0577999999999999</v>
-      </c>
-      <c r="J45" s="4" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A46" t="s">
-        <v>30</v>
-      </c>
-      <c r="B46" t="s">
-        <v>94</v>
-      </c>
-      <c r="C46" s="5" t="s">
-        <v>103</v>
-      </c>
-      <c r="D46" t="s">
-        <v>104</v>
-      </c>
-      <c r="E46" t="s">
-        <v>33</v>
-      </c>
-      <c r="F46">
-        <v>6</v>
-      </c>
-      <c r="G46" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="H46" s="1">
-        <f>3/100</f>
-        <v>0.03</v>
-      </c>
-      <c r="I46" s="1">
-        <f>Table1[[#This Row],[Qty]]*Table1[[#This Row],[Unit Cost]]</f>
-        <v>0.18</v>
-      </c>
-      <c r="J46" s="4" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="B47" t="s">
-        <v>94</v>
-      </c>
-      <c r="D47" t="s">
-        <v>106</v>
-      </c>
-      <c r="F47">
-        <v>1</v>
-      </c>
-      <c r="G47" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="H47" s="1">
-        <v>5</v>
-      </c>
-      <c r="I47" s="1">
-        <f>Table1[[#This Row],[Qty]]*Table1[[#This Row],[Unit Cost]]</f>
-        <v>5</v>
-      </c>
-      <c r="J47" s="4" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A48" t="s">
-        <v>43</v>
-      </c>
-      <c r="B48" t="s">
-        <v>108</v>
-      </c>
-      <c r="D48" t="s">
-        <v>109</v>
-      </c>
-      <c r="E48" t="s">
-        <v>110</v>
-      </c>
-      <c r="F48">
-        <v>1</v>
-      </c>
-      <c r="G48" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="H48" s="1">
-        <v>0</v>
-      </c>
-      <c r="I48" s="1">
-        <f>Table1[[#This Row],[Qty]]*Table1[[#This Row],[Unit Cost]]</f>
-        <v>0</v>
-      </c>
-      <c r="J48" s="6" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A49" t="s">
-        <v>30</v>
-      </c>
-      <c r="B49" t="s">
-        <v>108</v>
-      </c>
-      <c r="D49" t="s">
-        <v>112</v>
-      </c>
-      <c r="E49" t="s">
-        <v>33</v>
-      </c>
-      <c r="F49">
-        <v>2</v>
-      </c>
-      <c r="G49" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="H49" s="1">
-        <f>11.38/50</f>
-        <v>0.22760000000000002</v>
-      </c>
-      <c r="I49" s="1">
-        <f>Table1[[#This Row],[Qty]]*Table1[[#This Row],[Unit Cost]]</f>
-        <v>0.45520000000000005</v>
-      </c>
-      <c r="J49" s="4" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="B50" t="s">
-        <v>108</v>
-      </c>
-      <c r="D50" t="s">
-        <v>114</v>
-      </c>
-      <c r="E50" t="s">
-        <v>115</v>
-      </c>
-      <c r="F50">
-        <v>1</v>
-      </c>
-      <c r="G50" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="I50" s="1">
-        <f>Table1[[#This Row],[Qty]]*Table1[[#This Row],[Unit Cost]]</f>
-        <v>0</v>
-      </c>
-      <c r="J50" s="4" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="B51" t="s">
-        <v>108</v>
-      </c>
-      <c r="D51" t="s">
-        <v>117</v>
-      </c>
-      <c r="F51">
-        <v>1</v>
-      </c>
-      <c r="G51" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="I51" s="1">
-        <f>Table1[[#This Row],[Qty]]*Table1[[#This Row],[Unit Cost]]</f>
-        <v>0</v>
-      </c>
-      <c r="J51" s="6" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A52" t="s">
-        <v>30</v>
-      </c>
-      <c r="B52" t="s">
-        <v>108</v>
-      </c>
-      <c r="C52" s="5" t="s">
-        <v>119</v>
-      </c>
-      <c r="D52" t="s">
-        <v>120</v>
-      </c>
-      <c r="E52" t="s">
-        <v>33</v>
-      </c>
-      <c r="F52">
-        <v>3</v>
-      </c>
-      <c r="G52" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="H52" s="1">
-        <f>7.57/100</f>
-        <v>7.5700000000000003E-2</v>
-      </c>
-      <c r="I52" s="1">
-        <f>Table1[[#This Row],[Qty]]*Table1[[#This Row],[Unit Cost]]</f>
-        <v>0.22710000000000002</v>
-      </c>
-      <c r="J52" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A53" t="s">
-        <v>30</v>
-      </c>
-      <c r="B53" t="s">
-        <v>108</v>
-      </c>
-      <c r="C53" s="5" t="s">
-        <v>122</v>
-      </c>
-      <c r="D53" t="s">
-        <v>123</v>
-      </c>
-      <c r="E53" t="s">
-        <v>33</v>
-      </c>
-      <c r="F53">
-        <v>3</v>
-      </c>
-      <c r="G53" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="H53" s="1">
-        <f>7.41/100</f>
-        <v>7.4099999999999999E-2</v>
-      </c>
-      <c r="I53" s="1">
-        <f>Table1[[#This Row],[Qty]]*Table1[[#This Row],[Unit Cost]]</f>
-        <v>0.2223</v>
-      </c>
-      <c r="J53" s="4" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="B54" t="s">
-        <v>108</v>
-      </c>
-      <c r="C54" s="5" t="s">
-        <v>151</v>
-      </c>
-      <c r="D54" t="s">
-        <v>150</v>
-      </c>
-      <c r="E54" t="s">
-        <v>33</v>
-      </c>
-      <c r="F54">
-        <v>1</v>
-      </c>
-      <c r="G54" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="H54" s="7">
-        <v>4.95</v>
-      </c>
-      <c r="I54" s="7">
-        <f>Table1[[#This Row],[Qty]]*Table1[[#This Row],[Unit Cost]]</f>
-        <v>4.95</v>
-      </c>
-      <c r="J54" s="4" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="B55" t="s">
-        <v>125</v>
-      </c>
-      <c r="D55" t="s">
-        <v>126</v>
-      </c>
-      <c r="G55" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="I55" s="1">
-        <f>Table1[[#This Row],[Qty]]*Table1[[#This Row],[Unit Cost]]</f>
-        <v>0</v>
-      </c>
-      <c r="J55" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="B56" t="s">
-        <v>125</v>
-      </c>
-      <c r="D56" t="s">
-        <v>128</v>
-      </c>
-      <c r="F56">
-        <v>1</v>
-      </c>
-      <c r="G56" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="I56" s="1">
-        <f>Table1[[#This Row],[Qty]]*Table1[[#This Row],[Unit Cost]]</f>
-        <v>0</v>
-      </c>
-      <c r="J56" s="6" t="s">
-        <v>129</v>
-      </c>
-      <c r="K56" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="B57" t="s">
-        <v>125</v>
-      </c>
-      <c r="C57" s="5" t="s">
-        <v>131</v>
-      </c>
-      <c r="D57" t="s">
-        <v>132</v>
-      </c>
-      <c r="E57" t="s">
-        <v>133</v>
-      </c>
-      <c r="F57">
-        <v>1</v>
-      </c>
-      <c r="G57" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="H57" s="1">
-        <v>1.08</v>
-      </c>
-      <c r="I57" s="1">
-        <f>Table1[[#This Row],[Qty]]*Table1[[#This Row],[Unit Cost]]</f>
-        <v>1.08</v>
-      </c>
-      <c r="J57" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="B58" t="s">
-        <v>125</v>
-      </c>
-      <c r="D58" t="s">
-        <v>135</v>
-      </c>
-      <c r="G58" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="I58" s="1">
-        <f>Table1[[#This Row],[Qty]]*Table1[[#This Row],[Unit Cost]]</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A59" t="s">
-        <v>43</v>
-      </c>
-      <c r="B59" t="s">
-        <v>136</v>
-      </c>
-      <c r="C59" s="5" t="s">
-        <v>137</v>
-      </c>
-      <c r="D59" t="s">
-        <v>138</v>
-      </c>
-      <c r="E59" t="s">
-        <v>68</v>
-      </c>
-      <c r="F59">
-        <v>1</v>
-      </c>
-      <c r="G59" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="H59" s="1">
-        <v>1.49</v>
-      </c>
-      <c r="I59" s="1">
-        <f>Table1[[#This Row],[Qty]]*Table1[[#This Row],[Unit Cost]]</f>
-        <v>1.49</v>
-      </c>
-      <c r="J59" s="4" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="60" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A60" t="s">
-        <v>30</v>
-      </c>
-      <c r="B60" t="s">
-        <v>136</v>
-      </c>
-      <c r="C60" s="5" t="s">
-        <v>140</v>
-      </c>
-      <c r="D60" t="s">
-        <v>141</v>
-      </c>
-      <c r="E60" t="s">
-        <v>33</v>
-      </c>
-      <c r="F60">
-        <v>6</v>
-      </c>
-      <c r="G60" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="H60" s="1">
-        <f>8.44/100</f>
-        <v>8.4399999999999989E-2</v>
-      </c>
       <c r="I60" s="1">
         <f>Table1[[#This Row],[Qty]]*Table1[[#This Row],[Unit Cost]]</f>
-        <v>0.50639999999999996</v>
-      </c>
-      <c r="J60" s="4" t="s">
-        <v>142</v>
+        <v>0.18360000000000001</v>
       </c>
     </row>
     <row r="61" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="B61" t="s">
-        <v>136</v>
-      </c>
-      <c r="C61" s="5" t="s">
-        <v>91</v>
+        <v>135</v>
       </c>
       <c r="D61" t="s">
         <v>143</v>
       </c>
-      <c r="E61" t="s">
-        <v>33</v>
-      </c>
-      <c r="F61">
-        <v>6</v>
-      </c>
       <c r="G61" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="H61" s="1">
-        <f>3.06/100</f>
-        <v>3.0600000000000002E-2</v>
+        <v>22</v>
       </c>
       <c r="I61" s="1">
         <f>Table1[[#This Row],[Qty]]*Table1[[#This Row],[Unit Cost]]</f>
-        <v>0.18360000000000001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="62" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A62" t="s">
-        <v>43</v>
-      </c>
       <c r="B62" t="s">
-        <v>136</v>
+        <v>135</v>
+      </c>
+      <c r="C62" s="5" t="s">
+        <v>144</v>
       </c>
       <c r="D62" t="s">
-        <v>144</v>
+        <v>145</v>
+      </c>
+      <c r="E62" t="s">
+        <v>32</v>
+      </c>
+      <c r="F62">
+        <v>0.5</v>
       </c>
       <c r="G62" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
+      </c>
+      <c r="H62" s="1">
+        <v>9.65</v>
       </c>
       <c r="I62" s="1">
         <f>Table1[[#This Row],[Qty]]*Table1[[#This Row],[Unit Cost]]</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="B63" t="s">
-        <v>136</v>
-      </c>
-      <c r="C63" s="5" t="s">
-        <v>145</v>
-      </c>
-      <c r="D63" t="s">
+        <v>4.8250000000000002</v>
+      </c>
+      <c r="J62" t="s">
         <v>146</v>
       </c>
-      <c r="E63" t="s">
-        <v>33</v>
-      </c>
-      <c r="F63">
-        <v>0.5</v>
-      </c>
-      <c r="G63" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="H63" s="1">
-        <v>9.65</v>
-      </c>
-      <c r="I63" s="1">
-        <f>Table1[[#This Row],[Qty]]*Table1[[#This Row],[Unit Cost]]</f>
-        <v>4.8250000000000002</v>
-      </c>
-      <c r="J63" t="s">
+      <c r="K62" t="s">
         <v>147</v>
-      </c>
-      <c r="K63" t="s">
-        <v>148</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="J11" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
-    <hyperlink ref="J12" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
-    <hyperlink ref="J13" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
-    <hyperlink ref="J15" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
-    <hyperlink ref="J16" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
-    <hyperlink ref="J19" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
-    <hyperlink ref="J20" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
-    <hyperlink ref="J21" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
-    <hyperlink ref="J22" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
-    <hyperlink ref="J23" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
-    <hyperlink ref="J24" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
-    <hyperlink ref="J25" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
-    <hyperlink ref="J29" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
-    <hyperlink ref="J38" r:id="rId14" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
-    <hyperlink ref="J39" r:id="rId15" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
-    <hyperlink ref="J41" r:id="rId16" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
-    <hyperlink ref="J42" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
-    <hyperlink ref="J43" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
-    <hyperlink ref="J45" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
-    <hyperlink ref="J46" r:id="rId20" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
-    <hyperlink ref="J47" r:id="rId21" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
-    <hyperlink ref="J48" r:id="rId22" xr:uid="{00000000-0004-0000-0000-000015000000}"/>
-    <hyperlink ref="J49" r:id="rId23" xr:uid="{00000000-0004-0000-0000-000016000000}"/>
-    <hyperlink ref="J51" r:id="rId24" xr:uid="{00000000-0004-0000-0000-000017000000}"/>
-    <hyperlink ref="J53" r:id="rId25" xr:uid="{00000000-0004-0000-0000-000018000000}"/>
-    <hyperlink ref="J56" r:id="rId26" xr:uid="{00000000-0004-0000-0000-000019000000}"/>
-    <hyperlink ref="J59" r:id="rId27" xr:uid="{00000000-0004-0000-0000-00001A000000}"/>
-    <hyperlink ref="J60" r:id="rId28" xr:uid="{00000000-0004-0000-0000-00001B000000}"/>
-    <hyperlink ref="J54" r:id="rId29" xr:uid="{E0F0E1BC-BF9F-EC41-B567-F34F9756DE29}"/>
+    <hyperlink ref="J10" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="J11" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="J12" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="J14" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="J15" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
+    <hyperlink ref="J18" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="J19" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
+    <hyperlink ref="J20" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="J21" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
+    <hyperlink ref="J22" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
+    <hyperlink ref="J23" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
+    <hyperlink ref="J24" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
+    <hyperlink ref="J28" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
+    <hyperlink ref="J37" r:id="rId14" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
+    <hyperlink ref="J38" r:id="rId15" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
+    <hyperlink ref="J40" r:id="rId16" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
+    <hyperlink ref="J41" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
+    <hyperlink ref="J42" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
+    <hyperlink ref="J44" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
+    <hyperlink ref="J45" r:id="rId20" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
+    <hyperlink ref="J46" r:id="rId21" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
+    <hyperlink ref="J47" r:id="rId22" xr:uid="{00000000-0004-0000-0000-000015000000}"/>
+    <hyperlink ref="J48" r:id="rId23" xr:uid="{00000000-0004-0000-0000-000016000000}"/>
+    <hyperlink ref="J50" r:id="rId24" xr:uid="{00000000-0004-0000-0000-000017000000}"/>
+    <hyperlink ref="J52" r:id="rId25" xr:uid="{00000000-0004-0000-0000-000018000000}"/>
+    <hyperlink ref="J55" r:id="rId26" xr:uid="{00000000-0004-0000-0000-000019000000}"/>
+    <hyperlink ref="J58" r:id="rId27" xr:uid="{00000000-0004-0000-0000-00001A000000}"/>
+    <hyperlink ref="J59" r:id="rId28" xr:uid="{00000000-0004-0000-0000-00001B000000}"/>
+    <hyperlink ref="J53" r:id="rId29" xr:uid="{E0F0E1BC-BF9F-EC41-B567-F34F9756DE29}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
Documentation cleanup, laser cutting file fix
* Converted real images from .png to .jpeg
* Converted BOM to .csv, moved it into assets folder, and linked in md text
* Updated laser cutting files
</commit_message>
<xml_diff>
--- a/Walking-Setup/G6-Integration-Bill-of-Materials.xlsx
+++ b/Walking-Setup/G6-Integration-Bill-of-Materials.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10719"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lehenbaueri/Documents/GitHub/Fly-Lab-Gear/Walking-Setup/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A04A191-27BF-7F49-95A7-8C52F28F758E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3E5C8D6-42D6-5142-A83B-334A4CBC9E0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1640" yWindow="660" windowWidth="27460" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="306" uniqueCount="151">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="307" uniqueCount="152">
   <si>
     <t>Name</t>
   </si>
@@ -275,9 +275,6 @@
     <t>Fly Holder</t>
   </si>
   <si>
-    <t>Micromanipulator</t>
-  </si>
-  <si>
     <t>Micromanipulator adapter plate</t>
   </si>
   <si>
@@ -486,6 +483,12 @@
   </si>
   <si>
     <t>5779K108</t>
+  </si>
+  <si>
+    <t>LD40 Micromanipulator</t>
+  </si>
+  <si>
+    <t>../Miscellaneous/Adapter_metric-imperial_manipulator/production/LD40_Adapter_3in.step</t>
   </si>
 </sst>
 </file>
@@ -1733,7 +1736,7 @@
         <v>79</v>
       </c>
       <c r="D35" t="s">
-        <v>80</v>
+        <v>150</v>
       </c>
       <c r="F35">
         <v>1</v>
@@ -1747,6 +1750,9 @@
       <c r="I35" s="1">
         <f>Table1[[#This Row],[Qty]]*Table1[[#This Row],[Unit Cost]]</f>
         <v>80</v>
+      </c>
+      <c r="J35" t="s">
+        <v>151</v>
       </c>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.2">
@@ -1754,7 +1760,7 @@
         <v>79</v>
       </c>
       <c r="D36" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E36" t="s">
         <v>39</v>
@@ -1775,7 +1781,7 @@
         <v>79</v>
       </c>
       <c r="D37" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="E37" t="s">
         <v>39</v>
@@ -1791,7 +1797,7 @@
         <v>0</v>
       </c>
       <c r="J37" s="6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.2">
@@ -1799,7 +1805,7 @@
         <v>79</v>
       </c>
       <c r="D38" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E38" t="s">
         <v>39</v>
@@ -1815,7 +1821,7 @@
         <v>0</v>
       </c>
       <c r="J38" s="6" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.2">
@@ -1823,7 +1829,7 @@
         <v>79</v>
       </c>
       <c r="D39" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F39">
         <v>1</v>
@@ -1844,10 +1850,10 @@
         <v>79</v>
       </c>
       <c r="C40" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="D40" t="s">
         <v>87</v>
-      </c>
-      <c r="D40" t="s">
-        <v>88</v>
       </c>
       <c r="E40" t="s">
         <v>32</v>
@@ -1867,7 +1873,7 @@
         <v>0.88900000000000001</v>
       </c>
       <c r="J40" s="4" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.2">
@@ -1878,10 +1884,10 @@
         <v>79</v>
       </c>
       <c r="C41" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="D41" t="s">
         <v>90</v>
-      </c>
-      <c r="D41" t="s">
-        <v>91</v>
       </c>
       <c r="E41" t="s">
         <v>32</v>
@@ -1901,24 +1907,24 @@
         <v>3.0600000000000002E-2</v>
       </c>
       <c r="J41" s="4" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
+        <v>92</v>
+      </c>
+      <c r="B42" t="s">
+        <v>92</v>
+      </c>
+      <c r="C42" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="B42" t="s">
-        <v>93</v>
-      </c>
-      <c r="C42" s="5" t="s">
+      <c r="D42" t="s">
         <v>94</v>
       </c>
-      <c r="D42" t="s">
+      <c r="E42" t="s">
         <v>95</v>
-      </c>
-      <c r="E42" t="s">
-        <v>96</v>
       </c>
       <c r="F42">
         <v>1</v>
@@ -1934,15 +1940,15 @@
         <v>229</v>
       </c>
       <c r="J42" s="4" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B43" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D43" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F43">
         <v>1</v>
@@ -1961,13 +1967,13 @@
         <v>29</v>
       </c>
       <c r="B44" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C44" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="D44" t="s">
         <v>99</v>
-      </c>
-      <c r="D44" t="s">
-        <v>100</v>
       </c>
       <c r="E44" t="s">
         <v>32</v>
@@ -1987,7 +1993,7 @@
         <v>1.0577999999999999</v>
       </c>
       <c r="J44" s="4" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.2">
@@ -1995,13 +2001,13 @@
         <v>29</v>
       </c>
       <c r="B45" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C45" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="D45" t="s">
         <v>102</v>
-      </c>
-      <c r="D45" t="s">
-        <v>103</v>
       </c>
       <c r="E45" t="s">
         <v>32</v>
@@ -2021,15 +2027,15 @@
         <v>0.18</v>
       </c>
       <c r="J45" s="4" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B46" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D46" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="F46">
         <v>1</v>
@@ -2045,7 +2051,7 @@
         <v>5</v>
       </c>
       <c r="J46" s="4" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.2">
@@ -2053,13 +2059,13 @@
         <v>42</v>
       </c>
       <c r="B47" t="s">
+        <v>106</v>
+      </c>
+      <c r="D47" t="s">
         <v>107</v>
       </c>
-      <c r="D47" t="s">
+      <c r="E47" t="s">
         <v>108</v>
-      </c>
-      <c r="E47" t="s">
-        <v>109</v>
       </c>
       <c r="F47">
         <v>1</v>
@@ -2075,7 +2081,7 @@
         <v>0</v>
       </c>
       <c r="J47" s="6" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.2">
@@ -2083,10 +2089,10 @@
         <v>29</v>
       </c>
       <c r="B48" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D48" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E48" t="s">
         <v>32</v>
@@ -2106,52 +2112,52 @@
         <v>0.45520000000000005</v>
       </c>
       <c r="J48" s="4" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="49" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B49" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D49" t="s">
+        <v>112</v>
+      </c>
+      <c r="E49" t="s">
         <v>113</v>
       </c>
-      <c r="E49" t="s">
+      <c r="F49">
+        <v>1</v>
+      </c>
+      <c r="G49" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="I49" s="1">
+        <f>Table1[[#This Row],[Qty]]*Table1[[#This Row],[Unit Cost]]</f>
+        <v>0</v>
+      </c>
+      <c r="J49" s="4" t="s">
         <v>114</v>
-      </c>
-      <c r="F49">
-        <v>1</v>
-      </c>
-      <c r="G49" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="I49" s="1">
-        <f>Table1[[#This Row],[Qty]]*Table1[[#This Row],[Unit Cost]]</f>
-        <v>0</v>
-      </c>
-      <c r="J49" s="4" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="50" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B50" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D50" t="s">
+        <v>115</v>
+      </c>
+      <c r="F50">
+        <v>1</v>
+      </c>
+      <c r="G50" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="I50" s="1">
+        <f>Table1[[#This Row],[Qty]]*Table1[[#This Row],[Unit Cost]]</f>
+        <v>0</v>
+      </c>
+      <c r="J50" s="6" t="s">
         <v>116</v>
-      </c>
-      <c r="F50">
-        <v>1</v>
-      </c>
-      <c r="G50" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="I50" s="1">
-        <f>Table1[[#This Row],[Qty]]*Table1[[#This Row],[Unit Cost]]</f>
-        <v>0</v>
-      </c>
-      <c r="J50" s="6" t="s">
-        <v>117</v>
       </c>
     </row>
     <row r="51" spans="1:11" x14ac:dyDescent="0.2">
@@ -2159,13 +2165,13 @@
         <v>29</v>
       </c>
       <c r="B51" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C51" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="D51" t="s">
         <v>118</v>
-      </c>
-      <c r="D51" t="s">
-        <v>119</v>
       </c>
       <c r="E51" t="s">
         <v>32</v>
@@ -2185,7 +2191,7 @@
         <v>0.22710000000000002</v>
       </c>
       <c r="J51" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="52" spans="1:11" x14ac:dyDescent="0.2">
@@ -2193,13 +2199,13 @@
         <v>29</v>
       </c>
       <c r="B52" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C52" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="D52" t="s">
         <v>121</v>
-      </c>
-      <c r="D52" t="s">
-        <v>122</v>
       </c>
       <c r="E52" t="s">
         <v>32</v>
@@ -2219,18 +2225,18 @@
         <v>0.2223</v>
       </c>
       <c r="J52" s="4" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="53" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B53" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C53" s="5" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="D53" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="E53" t="s">
         <v>32</v>
@@ -2249,63 +2255,63 @@
         <v>4.95</v>
       </c>
       <c r="J53" s="4" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="54" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B54" t="s">
+        <v>123</v>
+      </c>
+      <c r="D54" t="s">
         <v>124</v>
       </c>
-      <c r="D54" t="s">
+      <c r="G54" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="I54" s="1">
+        <f>Table1[[#This Row],[Qty]]*Table1[[#This Row],[Unit Cost]]</f>
+        <v>0</v>
+      </c>
+      <c r="J54" t="s">
         <v>125</v>
-      </c>
-      <c r="G54" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="I54" s="1">
-        <f>Table1[[#This Row],[Qty]]*Table1[[#This Row],[Unit Cost]]</f>
-        <v>0</v>
-      </c>
-      <c r="J54" t="s">
-        <v>126</v>
       </c>
     </row>
     <row r="55" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B55" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D55" t="s">
+        <v>126</v>
+      </c>
+      <c r="F55">
+        <v>1</v>
+      </c>
+      <c r="G55" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="I55" s="1">
+        <f>Table1[[#This Row],[Qty]]*Table1[[#This Row],[Unit Cost]]</f>
+        <v>0</v>
+      </c>
+      <c r="J55" s="6" t="s">
         <v>127</v>
       </c>
-      <c r="F55">
-        <v>1</v>
-      </c>
-      <c r="G55" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="I55" s="1">
-        <f>Table1[[#This Row],[Qty]]*Table1[[#This Row],[Unit Cost]]</f>
-        <v>0</v>
-      </c>
-      <c r="J55" s="6" t="s">
+      <c r="K55" t="s">
         <v>128</v>
-      </c>
-      <c r="K55" t="s">
-        <v>129</v>
       </c>
     </row>
     <row r="56" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B56" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C56" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="D56" t="s">
         <v>130</v>
       </c>
-      <c r="D56" t="s">
+      <c r="E56" t="s">
         <v>131</v>
-      </c>
-      <c r="E56" t="s">
-        <v>132</v>
       </c>
       <c r="F56">
         <v>1</v>
@@ -2321,15 +2327,15 @@
         <v>1.08</v>
       </c>
       <c r="J56" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="57" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B57" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D57" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="G57" s="5" t="s">
         <v>22</v>
@@ -2344,13 +2350,13 @@
         <v>42</v>
       </c>
       <c r="B58" t="s">
+        <v>134</v>
+      </c>
+      <c r="C58" s="5" t="s">
         <v>135</v>
       </c>
-      <c r="C58" s="5" t="s">
+      <c r="D58" t="s">
         <v>136</v>
-      </c>
-      <c r="D58" t="s">
-        <v>137</v>
       </c>
       <c r="E58" t="s">
         <v>67</v>
@@ -2369,7 +2375,7 @@
         <v>1.49</v>
       </c>
       <c r="J58" s="4" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="59" spans="1:11" x14ac:dyDescent="0.2">
@@ -2377,13 +2383,13 @@
         <v>29</v>
       </c>
       <c r="B59" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C59" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="D59" t="s">
         <v>139</v>
-      </c>
-      <c r="D59" t="s">
-        <v>140</v>
       </c>
       <c r="E59" t="s">
         <v>32</v>
@@ -2403,7 +2409,7 @@
         <v>0.50639999999999996</v>
       </c>
       <c r="J59" s="4" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="60" spans="1:11" x14ac:dyDescent="0.2">
@@ -2411,13 +2417,13 @@
         <v>29</v>
       </c>
       <c r="B60" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C60" s="5" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D60" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E60" t="s">
         <v>32</v>
@@ -2442,10 +2448,10 @@
         <v>42</v>
       </c>
       <c r="B61" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D61" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="G61" s="5" t="s">
         <v>22</v>
@@ -2457,13 +2463,13 @@
     </row>
     <row r="62" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B62" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C62" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="D62" t="s">
         <v>144</v>
-      </c>
-      <c r="D62" t="s">
-        <v>145</v>
       </c>
       <c r="E62" t="s">
         <v>32</v>
@@ -2482,10 +2488,10 @@
         <v>4.8250000000000002</v>
       </c>
       <c r="J62" t="s">
+        <v>145</v>
+      </c>
+      <c r="K62" t="s">
         <v>146</v>
-      </c>
-      <c r="K62" t="s">
-        <v>147</v>
       </c>
     </row>
   </sheetData>

</xml_diff>